<commit_message>
fix(reports): mirror client payment status template
</commit_message>
<xml_diff>
--- a/docs/quality/golden-reports/billing-schedule-xlsx.xlsx
+++ b/docs/quality/golden-reports/billing-schedule-xlsx.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Billing &amp; Collection Register" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tenants Payment's Status Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Billing &amp; Collection Register'!$A$5:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tenants Payment''s Status Report'!$A$5:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -479,24 +479,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Billing &amp; Collection Register</t>
+          <t>Tenants Payment's Status Report</t>
         </is>
       </c>
     </row>
@@ -510,7 +511,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by admin · Generated 14 Aug 2026 10:35</t>
+          <t>Prepared by admin · Generated 14 Aug 2026 16:41</t>
         </is>
       </c>
     </row>
@@ -522,42 +523,47 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Unit / no.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Billing period</t>
+          <t>Rent / month</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Payment mode</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Billings up to</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Total billed</t>
+          <t>Balance B/F</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Current billings</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Outstanding</t>
+          <t>Total billings</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Receipts</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Outstanding C/F</t>
         </is>
       </c>
     </row>
@@ -572,30 +578,35 @@
           <t>101</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Jul 2026</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
+      <c r="C6" s="6" t="n">
         <v>185000</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
         <v>0</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>185000</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>185000</v>
       </c>
       <c r="H6" s="6" t="n">
+        <v>185000</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>185000</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n">
         <v>0</v>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>paid</t>
-        </is>
       </c>
     </row>
     <row r="7">
@@ -609,34 +620,39 @@
           <t>102</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Jul 2026</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="n">
+      <c r="C7" s="8" t="n">
         <v>120000</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="G7" s="8" t="n">
         <v>120000</v>
       </c>
-      <c r="G7" s="8" t="n">
-        <v>0</v>
-      </c>
       <c r="H7" s="8" t="n">
+        <v>120000</v>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>20000</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="n">
         <v>100000</v>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>overdue</t>
-        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I7"/>
+  <autoFilter ref="A5:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>